<commit_message>
Record four passing fan tests and TC05 finding
</commit_message>
<xml_diff>
--- a/Requirement_3_Physical_Product/04_Test_Cases_Excel/Senko_L1638_15_Test_Cases.xlsx
+++ b/Requirement_3_Physical_Product/04_Test_Cases_Excel/Senko_L1638_15_Test_Cases.xlsx
@@ -943,7 +943,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -1075,17 +1075,25 @@
       <c r="D4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>33</v>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Tờ giấy A5; băng dán; dụng cụ cố định giấy tại cùng vị trí cho các mức gió; ghi góc nâng của giấy theo từng mức.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>1) Tắt quạt, cố định tờ giấy tại cùng một vị trí trước quạt. 2) Bật lần lượt các mức tốc độ, giữ mỗi mức khoảng 15 giây. 3) Quan sát và ghi góc nâng của tờ giấy ở từng mức theo cùng một cách đo/ước lượng. 4) So sánh các góc nâng theo thứ tự mức tốc độ.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Góc nâng tờ giấy tăng theo các mức tốc độ; các mức liền kề có kết quả phân biệt được. Đây là tiêu chí so sánh nội bộ theo cùng cách bố trí, không phải ngưỡng lực gió do hãng công bố.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Theo số liệu người kiểm thử cung cấp, góc nâng tờ giấy ở ba mức tốc độ lần lượt là 45°, 50° và 70°. Các góc tăng theo mức tốc độ và phân biệt được từng mức.</t>
+        </is>
       </c>
       <c r="I4" s="2" t="s">
         <v>34</v>
@@ -1093,8 +1101,10 @@
       <c r="J4" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="K4" s="2" t="s">
-        <v>20</v>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Đã thay cách ghi khoảng cách trong bản AI bằng góc nâng theo dữ liệu thực tế. Phương pháp đo/ước lượng góc chưa được người kiểm thử mô tả.</t>
+        </is>
       </c>
     </row>
     <row r="5" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1113,14 +1123,20 @@
       <c r="E5" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>42</v>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>1) Bấm lần lượt các nút điều khiển và quan sát phản hồi. 2) Chọn một nút, bấm lặp 5 lần và đếm số lần phản hồi ngay. 3) Quan sát vị trí nút hoặc đèn báo nếu có để đối chiếu với trạng thái đang chọn.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Các nút được kiểm tra có phản hồi phù hợp với thao tác; nút được bấm lặp phải phản hồi ngay cả 5/5 lần. Đây là tiêu chí cho lượt thử đã thực hiện; không suy ra độ bền dài hạn.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Người kiểm thử xác nhận các nút đã thao tác phản hồi đúng trạng thái. Ở lượt bấm lặp, 5 lần nhấn đều phản hồi ngay (5/5).</t>
+        </is>
       </c>
       <c r="I5" s="2" t="s">
         <v>34</v>
@@ -1128,8 +1144,10 @@
       <c r="J5" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="K5" s="2" t="s">
-        <v>20</v>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Đã điều chỉnh số lần bấm lặp từ 10 của bản AI xuống 5 theo thực tế; kết quả 5/5 chỉ hỗ trợ kết luận cho 5 lần đã thử.</t>
+        </is>
       </c>
     </row>
     <row r="6" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1213,17 +1231,25 @@
       <c r="D8" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>67</v>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Nền phẳng cứng; giấy đặt dưới và phía trước đế tròn của quạt để quan sát dịch chuyển; không để giấy chạm lồng/cánh.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>1) Đặt quạt có đế tròn trên nền cứng phẳng; đặt giấy dưới và phía trước đế như bố trí thực tế. 2) Bật ở tốc độ cao nhất. 3) Quan sát liên tục khoảng 60 giây. 4) Ghi thân/đế có lắc, dịch chuyển không; giấy có xê dịch không; dây nguồn có bị kéo căng không. 5) Nếu có dịch chuyển, đo khoảng cách lớn nhất bằng thước.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Thân và đế quạt không lắc ngang hoặc di chuyển trên nền; giấy đặt dưới và phía trước đế không xê dịch; dây nguồn không bị kéo căng. Nếu có dịch chuyển thì ghi số đo; tiêu chí quan sát cho case này là không có dịch chuyển.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Người kiểm thử đặt giấy dưới và phía trước đế tròn, chạy quạt ở tốc độ cao nhất; giấy không dịch chuyển và quạt được xác nhận hoạt động ổn định. Không có số đo dịch chuyển riêng.</t>
+        </is>
       </c>
       <c r="I8" s="2" t="s">
         <v>34</v>
@@ -1231,8 +1257,10 @@
       <c r="J8" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="K8" s="2" t="s">
-        <v>69</v>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Đã sửa giả định ba chân trong test case AI cho đúng đế tròn của quạt thực tế; cách đặt giấy và quan sát theo người kiểm thử xác nhận.</t>
+        </is>
       </c>
     </row>
     <row r="9" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1455,8 +1483,10 @@
       <c r="G15" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="H15" s="2" t="s">
-        <v>117</v>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Người kiểm thử ngắt điện bằng cách rút phích rồi cắm lại; quạt tự chạy ổn định ở mức tốc độ đã chọn. Đây là kết quả quan sát được, nhưng cách ngắt/cấp điện khác Steps 3–4 dùng công tắc ngoài.</t>
+        </is>
       </c>
       <c r="I15" s="2" t="s">
         <v>34</v>
@@ -1464,8 +1494,10 @@
       <c r="J15" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="K15" s="2" t="s">
-        <v>110</v>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Theo người kiểm thử, kết quả hành vi là Pass; thao tác thực tế rút/cắm phích khác quy trình an toàn dự kiến. Không lặp lại thao tác này để quay bổ sung.</t>
+        </is>
       </c>
     </row>
     <row r="16" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1513,7 +1545,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -1574,22 +1606,30 @@
       <c r="A5" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>139</v>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Có chỉnh cao và chuyển hướng</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Chỉnh cao theo xác nhận người sở hữu; chuyển hướng đã kiểm ở TC05.</t>
+        </is>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>141</v>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Có hẹn giờ</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Người sở hữu xác nhận quạt có hẹn giờ; TC06 áp dụng nhưng chưa chạy.</t>
+        </is>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>